<commit_message>
added new fied "Comment"
</commit_message>
<xml_diff>
--- a/Requirments/SIQs.xlsx
+++ b/Requirments/SIQs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ITI\QA\Project\QA-project-tool\Requirments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F427BF40-393A-413E-8D4E-76176E886E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47C75D5-D106-48D0-8C8D-2F04390A3E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Question</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>Feature</t>
+  </si>
+  <si>
+    <t>Comment</t>
   </si>
 </sst>
 </file>
@@ -167,7 +170,34 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -479,6 +509,7 @@
     <col min="3" max="3" width="57" customWidth="1"/>
     <col min="4" max="4" width="45.42578125" customWidth="1"/>
     <col min="5" max="5" width="43.42578125" customWidth="1"/>
+    <col min="6" max="6" width="41.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="5" customFormat="1" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -497,7 +528,9 @@
       <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="4"/>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
@@ -523,6 +556,27 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E1:E1048576">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+      <formula>"Approved"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+      <formula>"N/A"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="7" operator="equal">
+      <formula>"In Disscusion"</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F1">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Approved"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Added SIQs in SIQ excel sheet
</commit_message>
<xml_diff>
--- a/Requirments/SIQs.xlsx
+++ b/Requirments/SIQs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21727"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ITI\QA\Project\QA-project-tool\Requirments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ITI_Courses\QA\QA-project-tool\Requirments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47C75D5-D106-48D0-8C8D-2F04390A3E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350F3CDF-DE65-4B73-8C87-B8374DA8E10C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t>Question</t>
   </si>
@@ -36,20 +36,291 @@
     <t>SIQ ID</t>
   </si>
   <si>
-    <t>Answer(Name,Date, Comment)</t>
-  </si>
-  <si>
-    <t>Feature</t>
-  </si>
-  <si>
-    <t>Comment</t>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Proposed answer</t>
+  </si>
+  <si>
+    <t>Customer answer</t>
+  </si>
+  <si>
+    <t>What are the login feature fields?</t>
+  </si>
+  <si>
+    <t>Register</t>
+  </si>
+  <si>
+    <t>What are the register feature fields?</t>
+  </si>
+  <si>
+    <r>
+      <t>Login feature fields are:
+ -</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Email </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Password fields</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+ -Link for user to register if not already registered
+ - Login button</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Home </t>
+  </si>
+  <si>
+    <t>What are the main features in home screen other than gallery of top travel destinations?</t>
+  </si>
+  <si>
+    <t>Unique user IDs</t>
+  </si>
+  <si>
+    <t>Module/Feature/Sub-feature</t>
+  </si>
+  <si>
+    <t>How shoud the unique user id get generated and how would it be used in the user flow?</t>
+  </si>
+  <si>
+    <t>User id is generated automatically upon user registration and is stored in database for user authentication during flight booking.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The home screen contains the following features:
+-Navigation bar with these nav links : Home, Gallery,book, about us
+-Search bar for user to search favored destinations
+-Gallery with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">few </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>top destinations and see more button that navigates to Gallery page with all touristic destinations
+-other customer reviews section</t>
+    </r>
+  </si>
+  <si>
+    <t>What happens upon user clicking a picture from the top travel destination gallery</t>
+  </si>
+  <si>
+    <t>Gallery</t>
+  </si>
+  <si>
+    <t>User is redirected to a page that shows the chosen travel destination details :
+-Descriptive picture of the destination
+-Destination name as title
+-Destination description
+-Reviews on the destination
+-Top places to visit for the destination
+-"Book now" button</t>
+  </si>
+  <si>
+    <t>Booking platform</t>
+  </si>
+  <si>
+    <t>Is there a feature that allows user to select flight destination and passenger count preferences ?</t>
+  </si>
+  <si>
+    <t>What is the user flow to book his flight?</t>
+  </si>
+  <si>
+    <t>Upon user clicking book now he/she is redirected to a page which has the following features:
+-toggling between one-way and round trips
+-From field for user to choose country he/she will travel from
+-To field for user to choose which country to travel to 
+- Adult passengers drop down for user to choose number of adults
+-Children number
+-Number of passengers with disabilities
+-Drop down for flight class (economy,business,etc..)
+-Search button</t>
+  </si>
+  <si>
+    <t>What is the required user flow to checkout the chosen flight?</t>
+  </si>
+  <si>
+    <t>Login-SIQ-01</t>
+  </si>
+  <si>
+    <t>Register-SIQ-02</t>
+  </si>
+  <si>
+    <t>Home-SIQ-03</t>
+  </si>
+  <si>
+    <t>UserID-SIQ-04</t>
+  </si>
+  <si>
+    <t>Gallery-SIQ-05</t>
+  </si>
+  <si>
+    <t>Book-SIQ-06</t>
+  </si>
+  <si>
+    <t>Book-SIQ-07</t>
+  </si>
+  <si>
+    <t>Book-SIQ-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Register feature fields are :
+-First name
+-Last name
+-Email
+-Password
+-Confirm password
+-Register button
+-Link to redirect user if already having an account to login
+-A confirmation email is sent to user mail box to activate his/her account
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upon user clikcing on search button for his flight preferences he is redirected to a page with the following features:
+-Airlines list with prices
+- Filter features: price , stops no. , Recommended, cheapest, fastest
+-sort by feature 
+</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Upon user clicking on the preferred airline, user is redirected to a page requiring passengers details:
+-First name
+-Last name
+-Gender
+-Date of birth 
+-Nationality 
+-Passport number and expiration date
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Then</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> another page to confirm user details upon user clicking on "continue" button.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>How user should pay for his flight?</t>
+  </si>
+  <si>
+    <t>Upon user clicking on confirm user is redirected to a page where he can enter card details:
+-Credit/debit card number
+-Cardholder name
+-Expiry date
+-Confirm payment button</t>
+  </si>
+  <si>
+    <t>Book-SIQ-09</t>
+  </si>
+  <si>
+    <t>Admin dashboard</t>
+  </si>
+  <si>
+    <t>Admin-SIQ-10</t>
+  </si>
+  <si>
+    <t>Rating system</t>
+  </si>
+  <si>
+    <t>Rating-SIQ-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Features include:
+-Registration and login features
+Overview section with:
+  -Customer count + Revenue calculation
+-Section for number of customers and option to view all customers
+-Charts for number of flights booked across a timeline
+Side panel with following navigation links:
+   -Home, income,etc.
+customer review
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It appears as a pop up window after customer successfully books and completes his/her payment which includes: 
+-review (star) rating 
+-review comment
+</t>
+  </si>
+  <si>
+    <t>Where should the rating system appear in the website?</t>
+  </si>
+  <si>
+    <t>What are the features of the admin dashboard?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76,6 +347,20 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -149,28 +434,58 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -501,20 +816,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AB12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.5703125" customWidth="1"/>
-    <col min="2" max="2" width="38.42578125" customWidth="1"/>
-    <col min="3" max="3" width="57" customWidth="1"/>
-    <col min="4" max="4" width="45.42578125" customWidth="1"/>
-    <col min="5" max="5" width="43.42578125" customWidth="1"/>
-    <col min="6" max="6" width="41.5703125" customWidth="1"/>
+    <col min="1" max="1" width="37.33203125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="38.44140625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="57" style="6" customWidth="1"/>
+    <col min="4" max="5" width="45.44140625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="41.5546875" style="6" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="5" customFormat="1" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" s="5" customFormat="1" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -523,13 +838,13 @@
         <v>0</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>1</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
@@ -554,36 +869,170 @@
       <c r="AA1" s="4"/>
       <c r="AB1" s="4"/>
     </row>
+    <row r="2" spans="1:28" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="126" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="122.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="209.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="156.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+  <phoneticPr fontId="5" type="noConversion"/>
+  <conditionalFormatting sqref="F1">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"Approved"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"N/A"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="7" operator="equal">
-      <formula>"In Disscusion"</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F1">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
-      <formula>"Approved"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>"N/A"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"In Disscusion"</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -598,10 +1047,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E1048576" xr:uid="{E5A70537-E00A-4E3C-8A84-DCB9E24EA7C9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1" xr:uid="{E5A70537-E00A-4E3C-8A84-DCB9E24EA7C9}">
       <formula1>"In Disscusion, Approved, N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>